<commit_message>
Restart item numbering at 1 each day, add day separator to export
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -55,7 +55,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -77,11 +77,25 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="medium">
+        <color rgb="002F4F4F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -96,6 +110,18 @@
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
@@ -1104,49 +1130,49 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="A17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>NFL Reebok T-Shirt</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>Blue</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
         <is>
           <t>XL Women's</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F17" s="7" t="inlineStr">
         <is>
           <t>Very good vintage condition</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G17" s="7" t="inlineStr">
         <is>
           <t>VWM - Women's Y2K Mix</t>
         </is>
       </c>
-      <c r="H17" s="4" t="n">
+      <c r="H17" s="8" t="n">
         <v>17.99</v>
       </c>
-      <c r="I17" s="5" t="n">
+      <c r="I17" s="9" t="n">
         <v>46252</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
@@ -1187,7 +1213,7 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
@@ -1224,7 +1250,7 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
@@ -1261,7 +1287,7 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
@@ -1298,7 +1324,7 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add 18 Aug items 7-8: Carhartt tee and Birkenstock sandals
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1359,8 +1359,82 @@
         <v>46252</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Carhartt T-Shirt</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Small Women's (4-6)</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="I23" s="5" t="n">
+        <v>46252</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Birkenstock Thong Sandals</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Natural</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Very good vintage condition</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>SF - Birkenstock</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>27.99</v>
+      </c>
+      <c r="I24" s="5" t="n">
+        <v>46252</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I22"/>
+  <autoFilter ref="A1:I24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 19 Aug item 1: orange Athletics women's t-shirt
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1433,8 +1433,49 @@
         <v>46252</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Athletics Women's T-Shirt</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Slight discrepancy on the back of the neck, barely noticeable (see images)</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>Very good vintage condition</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="n">
+        <v>12.99</v>
+      </c>
+      <c r="I25" s="9" t="n">
+        <v>46253</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I24"/>
+  <autoFilter ref="A1:I25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 19 Aug item 2: pink Ralph Lauren women's shirt, price pending
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1474,8 +1474,47 @@
         <v>46253</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Ralph Lauren Women's Shirt</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Pink</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr"/>
+      <c r="I26" s="5" t="n">
+        <v>46253</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I25"/>
+  <autoFilter ref="A1:I26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Set 19 Aug item 2 price to £18.00
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -1508,7 +1508,9 @@
           <t>VWM - Women's Y2K Mix</t>
         </is>
       </c>
-      <c r="H26" s="4" t="inlineStr"/>
+      <c r="H26" s="4" t="n">
+        <v>18</v>
+      </c>
       <c r="I26" s="5" t="n">
         <v>46253</v>
       </c>

</xml_diff>

<commit_message>
Add 19 Aug item 3: Chicago Bulls vest, size and price provisional
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1515,8 +1515,45 @@
         <v>46253</v>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Chicago Bulls Vest</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>16 (marked on label - men's/women's unconfirmed)</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="I27" s="5" t="n">
+        <v>46253</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I26"/>
+  <autoFilter ref="A1:I27"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 19 Aug item 4: red Ralph Lauren long sleeve tee
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1552,8 +1552,45 @@
         <v>46253</v>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Ralph Lauren Women's Long Sleeve T-Shirt</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Small (8)</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="I28" s="5" t="n">
+        <v>46253</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I27"/>
+  <autoFilter ref="A1:I28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 19 Aug item 5: NFL Broncos top, good condition
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1589,8 +1589,41 @@
         <v>46253</v>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>NFL Broncos Top</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Youth 18 (XXL) - translates to approx. women's Large</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Good condition</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="I29" s="5" t="n">
+        <v>46253</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I28"/>
+  <autoFilter ref="A1:I29"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 19 Aug item 6: black Ralph Lauren polo, price flagged as outlier
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1622,8 +1622,45 @@
         <v>46253</v>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Ralph Lauren Polo</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Small Men's</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>VWM - RL Lacoste Polos</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="n">
+        <v>30.99</v>
+      </c>
+      <c r="I30" s="5" t="n">
+        <v>46253</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I29"/>
+  <autoFilter ref="A1:I30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 19 Aug item 7: green Ralph Lauren polo
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1659,8 +1659,49 @@
         <v>46253</v>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Ralph Lauren Polo</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Large Men's</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>VWM - RL Lacoste Polos</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="I31" s="5" t="n">
+        <v>46253</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I30"/>
+  <autoFilter ref="A1:I31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 19 Aug item 8: blue Ralph Lauren polo with small back defect
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$32</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1700,8 +1700,49 @@
         <v>46253</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Ralph Lauren Polo</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Very small discrepancy on the back (see images)</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Medium Men's</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Very good vintage condition</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>VWM - RL Lacoste Polos</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="n">
+        <v>13.99</v>
+      </c>
+      <c r="I32" s="5" t="n">
+        <v>46253</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I31"/>
+  <autoFilter ref="A1:I32"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 19 Aug item 9: grey Ralph Lauren polo with front defect
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$33</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1741,8 +1741,49 @@
         <v>46253</v>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Ralph Lauren Polo</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Grey</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Slight discrepancy on the front</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Very good vintage condition</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>VWM - RL Lacoste Polos</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="n">
+        <v>12.99</v>
+      </c>
+      <c r="I33" s="5" t="n">
+        <v>46253</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I32"/>
+  <autoFilter ref="A1:I33"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 19 Aug item 10: navy Ralph Lauren polo
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1782,8 +1782,45 @@
         <v>46253</v>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Ralph Lauren Polo</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Navy</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr"/>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Small Men's</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>VWM - RL Lacoste Polos</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="I34" s="5" t="n">
+        <v>46253</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I33"/>
+  <autoFilter ref="A1:I34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 19 Aug item 11: Burberry Brit polo, price researched
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1819,8 +1819,41 @@
         <v>46253</v>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Burberry Brit Polo Shirt</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Slight marks on the front</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr"/>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>Good condition</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>SF - Men's Summer Designer Mix</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="I35" s="5" t="n">
+        <v>46253</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I34"/>
+  <autoFilter ref="A1:I35"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 19 Aug item 12: Cinema Etoile camisole, identified and priced
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$36</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1852,8 +1852,41 @@
         <v>46253</v>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Cinema Etoile Camisole/Chemise</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr"/>
+      <c r="D36" s="3" t="inlineStr"/>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Small Women's</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="I36" s="5" t="n">
+        <v>46253</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I35"/>
+  <autoFilter ref="A1:I36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 19 Aug item 13: Adidas women's fleece jacket, size and price researched
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$37</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1885,8 +1885,45 @@
         <v>46253</v>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Adidas Women's Jacket</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Fleece bottom</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>14 (UK women's - equivalent to Large)</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Good condition</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="n">
+        <v>22.99</v>
+      </c>
+      <c r="I37" s="5" t="n">
+        <v>46253</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I36"/>
+  <autoFilter ref="A1:I37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 19 Aug items 14-15: lace nightwear set and Buffalo Bills top
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1922,8 +1922,70 @@
         <v>46253</v>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Women's Lace Nightwear Set</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Blue lace</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr"/>
+      <c r="E38" s="3" t="inlineStr"/>
+      <c r="F38" s="3" t="inlineStr"/>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="n">
+        <v>12.99</v>
+      </c>
+      <c r="I38" s="5" t="n">
+        <v>46253</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Buffalo Bills Wild West Top</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr"/>
+      <c r="D39" s="3" t="inlineStr"/>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Large Women's</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="n">
+        <v>18.99</v>
+      </c>
+      <c r="I39" s="5" t="n">
+        <v>46253</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I37"/>
+  <autoFilter ref="A1:I39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 19 Aug item 16: Juicy Couture black cardigan
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1984,8 +1984,45 @@
         <v>46253</v>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Juicy Couture Cardigan</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr"/>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>XL Women's</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="I40" s="5" t="n">
+        <v>46253</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I39"/>
+  <autoFilter ref="A1:I40"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 19 Aug item 17: Dominique longline bridal bra, identified and priced
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2021,8 +2021,45 @@
         <v>46253</v>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Dominique Longline Bridal Bra (Bustier)</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr"/>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>44DD/E</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="n">
+        <v>16.99</v>
+      </c>
+      <c r="I41" s="5" t="n">
+        <v>46253</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I40"/>
+  <autoFilter ref="A1:I41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 19 Aug item 18: pink Juicy Couture top, price provisional pending fabric
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2058,8 +2058,45 @@
         <v>46253</v>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Juicy Couture Women's Top</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Pink</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr"/>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="I42" s="5" t="n">
+        <v>46253</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I41"/>
+  <autoFilter ref="A1:I42"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 19 Aug item 19: Carhartt women's tee with front speckles
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$43</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2095,8 +2095,49 @@
         <v>46253</v>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Carhartt Women's T-Shirt</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Green/mint, 100% cotton</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Slight speckles on the front</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>Small (4-6)</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>Good condition</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="I43" s="5" t="n">
+        <v>46253</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I42"/>
+  <autoFilter ref="A1:I43"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 19 Aug item 20: black Ralph Lauren women's polo
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2136,8 +2136,45 @@
         <v>46253</v>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Ralph Lauren Women's Polo Shirt</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Black with red pony</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr"/>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Medium (10-12) - classic fit</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H44" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="I44" s="5" t="n">
+        <v>46253</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I43"/>
+  <autoFilter ref="A1:I44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 19 Aug item 21: lilac Ralph Lauren Sport women's shirt
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$45</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2173,8 +2173,45 @@
         <v>46253</v>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Ralph Lauren Sport Women's Shirt</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Lilac purple</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr"/>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="I45" s="5" t="n">
+        <v>46253</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I44"/>
+  <autoFilter ref="A1:I45"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 19 Aug item 22: bronze/nude Birkenstocks size 37
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$46</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2210,8 +2210,45 @@
         <v>46253</v>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Birkenstocks</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>Bronze/nude</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr"/>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>37 (240mm)</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>Very good vintage condition</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>SF - Birkenstock</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="n">
+        <v>27.99</v>
+      </c>
+      <c r="I46" s="5" t="n">
+        <v>46253</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I45"/>
+  <autoFilter ref="A1:I46"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 19 Aug item 23: Birkenstock sandals with worn footbed
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$47</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2247,8 +2247,45 @@
         <v>46253</v>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Birkenstock Sandals</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr"/>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>Inner footbed a bit worn - exterior sole is in good condition. Would otherwise be very good condition</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>38 (245mm)</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>Good condition</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>SF - Birkenstock</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="I47" s="5" t="n">
+        <v>46253</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I46"/>
+  <autoFilter ref="A1:I47"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 19 Aug item 24: second pair of size 38 Birkenstocks
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$48</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2284,8 +2284,41 @@
         <v>46253</v>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Birkenstock Sandals</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr"/>
+      <c r="D48" s="3" t="inlineStr"/>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>38 (245mm)</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>Good condition</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>SF - Birkenstock</t>
+        </is>
+      </c>
+      <c r="H48" s="4" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="I48" s="5" t="n">
+        <v>46253</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I47"/>
+  <autoFilter ref="A1:I48"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 19 Aug item 25: yellow Birkenstocks size 36
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$49</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2317,8 +2317,45 @@
         <v>46253</v>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Birkenstocks</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Yellow</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr"/>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>36 (230mm)</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>Good condition</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>SF - Birkenstock</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="I49" s="5" t="n">
+        <v>46253</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I48"/>
+  <autoFilter ref="A1:I49"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Resolve 19 Aug items 6 and 18: correct polo price, confirm velour Juicy top
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -1653,7 +1653,7 @@
         </is>
       </c>
       <c r="H30" s="4" t="n">
-        <v>30.99</v>
+        <v>13.99</v>
       </c>
       <c r="I30" s="5" t="n">
         <v>46253</v>
@@ -2064,12 +2064,12 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Juicy Couture Women's Top</t>
+          <t>Juicy Couture Velour Top</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Pink</t>
+          <t>Pink velour</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr"/>
@@ -2089,7 +2089,7 @@
         </is>
       </c>
       <c r="H42" s="4" t="n">
-        <v>19.99</v>
+        <v>34.99</v>
       </c>
       <c r="I42" s="5" t="n">
         <v>46253</v>

</xml_diff>

<commit_message>
Set blank-defects-means-none rule, complete blue lace set and Burberry size
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -560,7 +560,11 @@
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr"/>
-      <c r="D2" s="3" t="inlineStr"/>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Large Women's</t>
@@ -597,7 +601,11 @@
           <t>Navy with pinstripes</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
           <t>XXL</t>
@@ -630,7 +638,11 @@
           <t>Tartan check, labels cut</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Small Men's</t>
@@ -667,7 +679,11 @@
           <t>Black</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Large Women's</t>
@@ -786,7 +802,11 @@
           <t>Navy</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr"/>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
           <t>Medium (10-12)</t>
@@ -823,7 +843,11 @@
           <t>Green</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
           <t>Large (oversized fit)</t>
@@ -1106,7 +1130,11 @@
           <t>Turquoise</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
           <t>Large</t>
@@ -1262,7 +1290,11 @@
           <t>Blue</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
           <t>Large Women's</t>
@@ -1299,7 +1331,11 @@
           <t>Dark navy blue, Walter Payton number 34 on the front</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
           <t>XL Women's</t>
@@ -1336,7 +1372,11 @@
           <t>Turquoise</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr"/>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
           <t>Large</t>
@@ -1369,7 +1409,11 @@
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr"/>
-      <c r="D23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
           <t>Small Women's (4-6)</t>
@@ -1529,7 +1573,11 @@
           <t>Red</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
           <t>16 (marked on label - men's/women's unconfirmed)</t>
@@ -1566,7 +1614,11 @@
           <t>Red</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr"/>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
           <t>Small (8)</t>
@@ -1599,7 +1651,11 @@
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr"/>
-      <c r="D29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
           <t>Youth 18 (XXL) - translates to approx. women's Large</t>
@@ -1636,7 +1692,11 @@
           <t>Black</t>
         </is>
       </c>
-      <c r="D30" s="3" t="inlineStr"/>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
           <t>Small Men's</t>
@@ -1796,7 +1856,11 @@
           <t>Navy</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr"/>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
           <t>Small Men's</t>
@@ -1834,7 +1898,11 @@
           <t>Slight marks on the front</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr"/>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
           <t>Good condition</t>
@@ -1862,7 +1930,11 @@
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr"/>
-      <c r="D36" s="3" t="inlineStr"/>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
           <t>Small Women's</t>
@@ -1899,7 +1971,11 @@
           <t>Fleece bottom</t>
         </is>
       </c>
-      <c r="D37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
           <t>14 (UK women's - equivalent to Large)</t>
@@ -1928,7 +2004,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Women's Lace Nightwear Set</t>
+          <t>Women's Lace Babydoll Set</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -1936,9 +2012,21 @@
           <t>Blue lace</t>
         </is>
       </c>
-      <c r="D38" s="3" t="inlineStr"/>
-      <c r="E38" s="3" t="inlineStr"/>
-      <c r="F38" s="3" t="inlineStr"/>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Small Women's</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
           <t>VWM - Women's Y2K Mix</t>
@@ -1961,7 +2049,11 @@
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr"/>
-      <c r="D39" s="3" t="inlineStr"/>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
           <t>Large Women's</t>
@@ -1998,7 +2090,11 @@
           <t>Black</t>
         </is>
       </c>
-      <c r="D40" s="3" t="inlineStr"/>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
           <t>XL Women's</t>
@@ -2035,7 +2131,11 @@
           <t>White</t>
         </is>
       </c>
-      <c r="D41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
           <t>44DD/E</t>
@@ -2072,7 +2172,11 @@
           <t>Pink velour</t>
         </is>
       </c>
-      <c r="D42" s="3" t="inlineStr"/>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
           <t>Medium</t>
@@ -2150,7 +2254,11 @@
           <t>Black with red pony</t>
         </is>
       </c>
-      <c r="D44" s="3" t="inlineStr"/>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
           <t>Medium (10-12) - classic fit</t>
@@ -2187,7 +2295,11 @@
           <t>Lilac purple</t>
         </is>
       </c>
-      <c r="D45" s="3" t="inlineStr"/>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
           <t>Small</t>
@@ -2224,7 +2336,11 @@
           <t>Bronze/nude</t>
         </is>
       </c>
-      <c r="D46" s="3" t="inlineStr"/>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
           <t>37 (240mm)</t>
@@ -2294,7 +2410,11 @@
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr"/>
-      <c r="D48" s="3" t="inlineStr"/>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
           <t>38 (245mm)</t>
@@ -2331,7 +2451,11 @@
           <t>Yellow</t>
         </is>
       </c>
-      <c r="D49" s="3" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
           <t>36 (230mm)</t>

</xml_diff>

<commit_message>
Start new day: add 20 Aug item 1, orange Adidas hoodie
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$50</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2478,8 +2478,45 @@
         <v>46253</v>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>Adidas Hoodie</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>A few dark marks and discrepancies on the front (see images)</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>UK 30/32 (chest) - approx. women's XS-S</t>
+        </is>
+      </c>
+      <c r="F50" s="7" t="inlineStr"/>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H50" s="8" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="I50" s="9" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I49"/>
+  <autoFilter ref="A1:I50"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Set condition on 20 Aug item 1
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -2502,7 +2502,11 @@
           <t>UK 30/32 (chest) - approx. women's XS-S</t>
         </is>
       </c>
-      <c r="F50" s="7" t="inlineStr"/>
+      <c r="F50" s="7" t="inlineStr">
+        <is>
+          <t>Good condition</t>
+        </is>
+      </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
           <t>VWM - Women's Y2K Mix</t>

</xml_diff>

<commit_message>
Add 20 Aug item 2: Nike Georgia hoodie
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$51</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I50"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2519,8 +2519,45 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Nike Georgia Hoodie</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr"/>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>A few marks (see images)</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>Small Women's (4-6)</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>Very good vintage condition</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="I51" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I50"/>
+  <autoFilter ref="A1:I51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Move defects to bottom of description field, set rule in conventions
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -922,7 +922,8 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Navy</t>
+          <t>Navy
+One small discrepancy on the front (see images)</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -963,7 +964,8 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Black and navy</t>
+          <t>Black and navy
+White marks on right sleeve (see images)</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -1004,7 +1006,8 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Green with orange pony</t>
+          <t>Green with orange pony
+Discrepancies on the front</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -1045,7 +1048,8 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Light green</t>
+          <t>Light green
+Discrepancies on the front (see images)</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -1209,7 +1213,8 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Navy with an orange band and white</t>
+          <t>Navy with an orange band and white
+Marks on left sleeve (see images)</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -1488,7 +1493,8 @@
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Orange</t>
+          <t>Orange
+Slight discrepancy on the back of the neck, barely noticeable (see images)</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
@@ -1771,7 +1777,8 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Blue</t>
+          <t>Blue
+Very small discrepancy on the back (see images)</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -1812,7 +1819,8 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Grey</t>
+          <t>Grey
+Slight discrepancy on the front</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -1892,7 +1900,11 @@
           <t>Burberry Brit Polo Shirt</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr"/>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Slight marks on the front</t>
+        </is>
+      </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
           <t>Slight marks on the front</t>
@@ -2210,7 +2222,8 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Green/mint, 100% cotton</t>
+          <t>Green/mint, 100% cotton
+Slight speckles on the front</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -2372,7 +2385,11 @@
           <t>Birkenstock Sandals</t>
         </is>
       </c>
-      <c r="C47" s="3" t="inlineStr"/>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>Inner footbed a bit worn - exterior sole is in good condition. Would otherwise be very good condition</t>
+        </is>
+      </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
           <t>Inner footbed a bit worn - exterior sole is in good condition. Would otherwise be very good condition</t>
@@ -2489,7 +2506,8 @@
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>Orange</t>
+          <t>Orange
+A few dark marks and discrepancies on the front (see images)</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
@@ -2528,7 +2546,11 @@
           <t>Nike Georgia Hoodie</t>
         </is>
       </c>
-      <c r="C51" s="3" t="inlineStr"/>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>A few marks (see images)</t>
+        </is>
+      </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
           <t>A few marks (see images)</t>

</xml_diff>

<commit_message>
Add 20 Aug item 3: Ralph Lauren women's top, price pending
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$52</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2578,8 +2578,47 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Ralph Lauren Women's Top</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>100% cotton</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>Medium (12-14)</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>Good condition</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H52" s="4" t="inlineStr"/>
+      <c r="I52" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I51"/>
+  <autoFilter ref="A1:I52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 4: red Lacoste women's polo
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$53</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2617,8 +2617,49 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Lacoste Women's Polo</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>Small Women's</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>Good condition</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H53" s="4" t="n">
+        <v>11.99</v>
+      </c>
+      <c r="I53" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I52"/>
+  <autoFilter ref="A1:I53"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add defects to 20 Aug item 4 and revise price to £9.99
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -2628,12 +2628,13 @@
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Red</t>
+          <t>Red
+Marks and discrepancies on the back and front, mainly on the back</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Marks and discrepancies on the back and front, mainly on the back</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
@@ -2652,7 +2653,7 @@
         </is>
       </c>
       <c r="H53" s="4" t="n">
-        <v>11.99</v>
+        <v>9.99</v>
       </c>
       <c r="I53" s="5" t="n">
         <v>46254</v>

</xml_diff>

<commit_message>
Add 20 Aug item 5: Juicy Couture black blouse, size researched
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$54</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2659,8 +2659,49 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Juicy Couture Blouse</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>2 (likely US 2 = UK 6 / XS - unconfirmed)</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H54" s="4" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="I54" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I53"/>
+  <autoFilter ref="A1:I54"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 6: pink North Face fleece
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$55</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I54"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2700,8 +2700,49 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>The North Face Fleece</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>Pink</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="I55" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I54"/>
+  <autoFilter ref="A1:I55"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 7: Juicy Couture track jacket
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$56</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2741,8 +2741,45 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Juicy Couture Track Jacket</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr"/>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H56" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="I56" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I55"/>
+  <autoFilter ref="A1:I56"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 8: Lululemon women's top
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$57</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I56"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2778,8 +2778,45 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Lululemon Women's Top</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr"/>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>Small Women's (no size label - owner's estimate, unconfirmed)</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="n">
+        <v>22.99</v>
+      </c>
+      <c r="I57" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I56"/>
+  <autoFilter ref="A1:I57"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 9: North Face zip-up fleece
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$58</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I57"/>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2815,8 +2815,49 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>The North Face Zip-Up Fleece</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>Small discrepancies on the arm, barely noticeable (see images)</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>Small discrepancies on the arm, barely noticeable (see images)</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>Very good vintage condition</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H58" s="4" t="n">
+        <v>12.99</v>
+      </c>
+      <c r="I58" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I57"/>
+  <autoFilter ref="A1:I58"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 10: burgundy Carhartt fleece, price pending
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$59</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I58"/>
+  <dimension ref="A1:I59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2856,8 +2856,47 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Carhartt Women's Fleece</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>Burgundy</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>XS (4-6) - relaxed fit</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>Very good vintage condition</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H59" s="4" t="inlineStr"/>
+      <c r="I59" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I58"/>
+  <autoFilter ref="A1:I59"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 11: brown Carhartt jumper
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$60</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2895,8 +2895,45 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Carhartt Jumper</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>Brown</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr"/>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H60" s="4" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="I60" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I59"/>
+  <autoFilter ref="A1:I60"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Price 20 Aug item 10 with fading noted
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -2867,7 +2867,7 @@
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Burgundy</t>
+          <t>Burgundy, slightly faded</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
@@ -2890,7 +2890,9 @@
           <t>VWM - Women's Y2K Mix</t>
         </is>
       </c>
-      <c r="H59" s="4" t="inlineStr"/>
+      <c r="H59" s="4" t="n">
+        <v>13.99</v>
+      </c>
       <c r="I59" s="5" t="n">
         <v>46254</v>
       </c>

</xml_diff>

<commit_message>
Add 20 Aug item 12: black nightwear chemise, identified and priced
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$61</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2934,8 +2934,49 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Women's Chemise (Nightwear)</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>Black, 83% nylon / 17% spandex</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>40D</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H61" s="4" t="n">
+        <v>12.99</v>
+      </c>
+      <c r="I61" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I60"/>
+  <autoFilter ref="A1:I61"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 13: women's shorts
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$62</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I61"/>
+  <dimension ref="A1:I62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2975,8 +2975,50 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>Women's Shorts</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>Light wash
+Slight marks to the front and a bit to the back</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>Slight marks to the front and a bit to the back</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>6 (31 waist, 12 leg)</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>Good condition</t>
+        </is>
+      </c>
+      <c r="G62" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H62" s="4" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="I62" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I61"/>
+  <autoFilter ref="A1:I62"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 14: Carhartt women's hoodie
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$63</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I62"/>
+  <dimension ref="A1:I63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3017,8 +3017,49 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Carhartt Women's Hoodie</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>Slight mark on the front (see images)</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>Slight mark on the front (see images)</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>Large - relaxed fit</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>Good condition</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H63" s="4" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="I63" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I62"/>
+  <autoFilter ref="A1:I63"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 15: Carhartt cream top, price blocked on garment type
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$64</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I63"/>
+  <dimension ref="A1:I64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3058,8 +3058,48 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>Carhartt Women's Top (garment type unconfirmed)</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>Cream
+A couple of unnoticeable marks on the front (see images)</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>A couple of unnoticeable marks on the front (see images)</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>Large (12-14) - relaxed fit</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>Very good vintage condition</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H64" s="4" t="inlineStr"/>
+      <c r="I64" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I63"/>
+  <autoFilter ref="A1:I64"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 16: Juicy Couture black cardigan
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$65</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:I65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3098,8 +3098,49 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>Juicy Couture Cardigan</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>Black, 80% cotton / 20% polyester</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>Large Women's</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H65" s="4" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="I65" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I64"/>
+  <autoFilter ref="A1:I65"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 17: Juicy Couture denim jacket
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$66</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I65"/>
+  <dimension ref="A1:I66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3139,8 +3139,41 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>Juicy Couture Denim Jacket</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr"/>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr"/>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G66" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H66" s="4" t="n">
+        <v>27.99</v>
+      </c>
+      <c r="I66" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I65"/>
+  <autoFilter ref="A1:I66"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 18: third black Juicy Couture cardigan
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$67</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I66"/>
+  <dimension ref="A1:I67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3172,8 +3172,49 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>Juicy Couture Cardigan</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H67" s="4" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="I67" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I66"/>
+  <autoFilter ref="A1:I67"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 19: Juicy Couture cashmere zip hoodie
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$68</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I67"/>
+  <dimension ref="A1:I68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3213,8 +3213,49 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>Juicy Couture Cashmere Zip-Up Hoodie</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>Dark grey, 100% cashmere</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H68" s="4" t="n">
+        <v>44.99</v>
+      </c>
+      <c r="I68" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I67"/>
+  <autoFilter ref="A1:I68"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 20: Val Mode burgundy nightwear, identified
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$69</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I68"/>
+  <dimension ref="A1:I69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3254,8 +3254,43 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>Val Mode Nightgown (exact type to confirm)</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>Burgundy</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr"/>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H69" s="4" t="inlineStr"/>
+      <c r="I69" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I68"/>
+  <autoFilter ref="A1:I69"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 21: Guess women's shorts
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$70</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I69"/>
+  <dimension ref="A1:I70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3289,8 +3289,44 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>Guess Women's Shorts</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>Natural tan, 100% cotton
+A couple of discrepancies (see images)</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>A couple of discrepancies (see images)</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>29 (waist)</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>Good condition</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="inlineStr"/>
+      <c r="H70" s="4" t="inlineStr"/>
+      <c r="I70" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I69"/>
+  <autoFilter ref="A1:I70"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 22: red Ralph Lauren cable knit jumper
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$71</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I70"/>
+  <dimension ref="A1:I71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3325,8 +3325,49 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>Ralph Lauren Cable Knit Jumper</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H71" s="4" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="I71" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I70"/>
+  <autoFilter ref="A1:I71"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 23: Rock Revival women's shorts
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$72</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I71"/>
+  <dimension ref="A1:I72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3366,8 +3366,44 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>Rock Revival Women's Shorts</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>Greeny turquoise
+Small discrepancy on the back, nothing too much (see images)</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>Small discrepancy on the back, nothing too much (see images)</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>24 (waist)</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>Very good vintage condition</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr"/>
+      <c r="H72" s="4" t="inlineStr"/>
+      <c r="I72" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I71"/>
+  <autoFilter ref="A1:I72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Set SKU on 20 Aug item 23
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -3396,7 +3396,11 @@
           <t>Very good vintage condition</t>
         </is>
       </c>
-      <c r="G72" s="3" t="inlineStr"/>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
       <c r="H72" s="4" t="inlineStr"/>
       <c r="I72" s="5" t="n">
         <v>46254</v>

</xml_diff>

<commit_message>
Add 20 Aug item 24: black skirt
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$73</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I72"/>
+  <dimension ref="A1:I73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3406,8 +3406,49 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>Yana Women's Skirt (brand to confirm)</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>Medium (waist not stated)</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G73" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H73" s="4" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="I73" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I72"/>
+  <autoFilter ref="A1:I73"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Set defects and SKU on 20 Aug item 21
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -3301,12 +3301,12 @@
       <c r="C70" s="3" t="inlineStr">
         <is>
           <t>Natural tan, 100% cotton
-A couple of discrepancies (see images)</t>
+Marks on front (see images)</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>A couple of discrepancies (see images)</t>
+          <t>Marks on front (see images)</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
@@ -3319,7 +3319,11 @@
           <t>Good condition</t>
         </is>
       </c>
-      <c r="G70" s="3" t="inlineStr"/>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
       <c r="H70" s="4" t="inlineStr"/>
       <c r="I70" s="5" t="n">
         <v>46254</v>

</xml_diff>

<commit_message>
Add 20 Aug item 25: corset, type and price pending identification
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$74</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I73"/>
+  <dimension ref="A1:I74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3451,8 +3451,39 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>Corset (item type and size to confirm)</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr"/>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr"/>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G74" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H74" s="4" t="inlineStr"/>
+      <c r="I74" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I73"/>
+  <autoFilter ref="A1:I74"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 26: black nylon/spandex dress
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$75</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I74"/>
+  <dimension ref="A1:I75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3482,8 +3482,49 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>Women's Dress</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>Black, nylon and spandex</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t>28/29</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G75" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H75" s="4" t="n">
+        <v>16.99</v>
+      </c>
+      <c r="I75" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I74"/>
+  <autoFilter ref="A1:I75"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 27: women's miniskirt
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$76</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I75"/>
+  <dimension ref="A1:I76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3523,8 +3523,49 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>Women's Miniskirt</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>One speckle of a mark on the back - indistinct and hard to notice (see images)</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>One speckle of a mark on the back - indistinct and hard to notice (see images)</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H76" s="4" t="n">
+        <v>13.99</v>
+      </c>
+      <c r="I76" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I75"/>
+  <autoFilter ref="A1:I76"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 28, identify Yana K brand and revise item 24
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$77</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I76"/>
+  <dimension ref="A1:I77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3416,7 +3416,7 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>Yana Women's Skirt (brand to confirm)</t>
+          <t>Yana K Women's Skirt</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
@@ -3445,7 +3445,7 @@
         </is>
       </c>
       <c r="H73" s="4" t="n">
-        <v>14.99</v>
+        <v>17.99</v>
       </c>
       <c r="I73" s="5" t="n">
         <v>46254</v>
@@ -3564,8 +3564,49 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>Yana K Women's Miniskirt</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>96% cotton / 4% spandex</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G77" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H77" s="4" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="I77" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I76"/>
+  <autoFilter ref="A1:I77"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 29: Maidenform half slip
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$78</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I77"/>
+  <dimension ref="A1:I78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3605,8 +3605,45 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>Maidenform Half Slip (skirt or slip - to confirm)</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr"/>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H78" s="4" t="n">
+        <v>12.99</v>
+      </c>
+      <c r="I78" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I77"/>
+  <autoFilter ref="A1:I78"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 31: Urban Outfitters top, note missing item 30
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$79</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I78"/>
+  <dimension ref="A1:I79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3642,8 +3642,49 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>Urban Outfitters Women's Top</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>Dark burnt orange</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>Small (no size label - owner's estimate, unconfirmed)</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G79" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H79" s="4" t="n">
+        <v>12.99</v>
+      </c>
+      <c r="I79" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I78"/>
+  <autoFilter ref="A1:I79"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 30: Pendleton red cardigan
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$80</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I79"/>
+  <dimension ref="A1:I80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3644,16 +3644,16 @@
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>Urban Outfitters Women's Top</t>
+          <t>Pendleton Cardigan</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>Dark burnt orange</t>
+          <t>Red</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
@@ -3663,7 +3663,7 @@
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>Small (no size label - owner's estimate, unconfirmed)</t>
+          <t>12</t>
         </is>
       </c>
       <c r="F79" s="3" t="inlineStr">
@@ -3676,15 +3676,54 @@
           <t>VWM - Women's Y2K Mix</t>
         </is>
       </c>
-      <c r="H79" s="4" t="n">
-        <v>12.99</v>
-      </c>
+      <c r="H79" s="4" t="inlineStr"/>
       <c r="I79" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>Urban Outfitters Women's Top</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>Dark burnt orange</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>Small (no size label - owner's estimate, unconfirmed)</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G80" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H80" s="4" t="n">
+        <v>12.99</v>
+      </c>
+      <c r="I80" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I79"/>
+  <autoFilter ref="A1:I80"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 32: Vigoss denim shorts
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$81</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I80"/>
+  <dimension ref="A1:I81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3722,8 +3722,43 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>Vigoss Women's Denim Shorts</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr"/>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="inlineStr">
+        <is>
+          <t>15/16 (US junior sizing - approx. UK 16), 3.5in inseam</t>
+        </is>
+      </c>
+      <c r="F81" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G81" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H81" s="4" t="inlineStr"/>
+      <c r="I81" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I80"/>
+  <autoFilter ref="A1:I81"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 33: Calvin Klein tie
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$82</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I81"/>
+  <dimension ref="A1:I82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3757,8 +3757,49 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>Calvin Klein Tie</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>Purple</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>One size</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G82" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H82" s="4" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="I82" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I81"/>
+  <autoFilter ref="A1:I82"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 35: Ralph Lauren jumper, satisfactory grade
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$83</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I82"/>
+  <dimension ref="A1:I83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3798,8 +3798,46 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>Ralph Lauren Jumper</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>Orange, round neck
+Marks on the front (see images)</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>Marks on the front (see images)</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr">
+        <is>
+          <t>8-10</t>
+        </is>
+      </c>
+      <c r="F83" s="3" t="inlineStr">
+        <is>
+          <t>Satisfactory condition</t>
+        </is>
+      </c>
+      <c r="G83" s="3" t="inlineStr"/>
+      <c r="H83" s="4" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="I83" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I82"/>
+  <autoFilter ref="A1:I83"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 34: Birkenstock sandals size 34
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$84</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I83"/>
+  <dimension ref="A1:I84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3800,44 +3800,81 @@
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>Birkenstock Sandals</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>Inner footbed a bit worn with dark marks, believed to be water damage. Exterior: bottom soles, leather and cork all in very good condition</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>Inner footbed a bit worn with dark marks, believed to be water damage. Exterior: bottom soles, leather and cork all in very good condition</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="F83" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G83" s="3" t="inlineStr"/>
+      <c r="H83" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="I83" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="B83" s="3" t="inlineStr">
+      <c r="B84" s="3" t="inlineStr">
         <is>
           <t>Ralph Lauren Jumper</t>
         </is>
       </c>
-      <c r="C83" s="3" t="inlineStr">
+      <c r="C84" s="3" t="inlineStr">
         <is>
           <t>Orange, round neck
 Marks on the front (see images)</t>
         </is>
       </c>
-      <c r="D83" s="3" t="inlineStr">
+      <c r="D84" s="3" t="inlineStr">
         <is>
           <t>Marks on the front (see images)</t>
         </is>
       </c>
-      <c r="E83" s="3" t="inlineStr">
+      <c r="E84" s="3" t="inlineStr">
         <is>
           <t>8-10</t>
         </is>
       </c>
-      <c r="F83" s="3" t="inlineStr">
+      <c r="F84" s="3" t="inlineStr">
         <is>
           <t>Satisfactory condition</t>
         </is>
       </c>
-      <c r="G83" s="3" t="inlineStr"/>
-      <c r="H83" s="4" t="n">
+      <c r="G84" s="3" t="inlineStr"/>
+      <c r="H84" s="4" t="n">
         <v>9.99</v>
       </c>
-      <c r="I83" s="5" t="n">
+      <c r="I84" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I83"/>
+  <autoFilter ref="A1:I84"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Set standing rule: Birkenstock sandals always take SF - Birkenstock SKU
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -3827,7 +3827,11 @@
           <t>Very good condition</t>
         </is>
       </c>
-      <c r="G83" s="3" t="inlineStr"/>
+      <c r="G83" s="3" t="inlineStr">
+        <is>
+          <t>SF - Birkenstock</t>
+        </is>
+      </c>
       <c r="H83" s="4" t="n">
         <v>29.99</v>
       </c>

</xml_diff>

<commit_message>
Set SKU on 20 Aug item 35
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -3869,7 +3869,11 @@
           <t>Satisfactory condition</t>
         </is>
       </c>
-      <c r="G84" s="3" t="inlineStr"/>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
       <c r="H84" s="4" t="n">
         <v>9.99</v>
       </c>

</xml_diff>

<commit_message>
Add 20 Aug item 36: teal Nike track bottoms
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$85</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I84"/>
+  <dimension ref="A1:I85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3881,8 +3881,47 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>Nike Track Bottoms</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>Teal</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>Large (12-14) Women's</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G85" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H85" s="4" t="inlineStr"/>
+      <c r="I85" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I84"/>
+  <autoFilter ref="A1:I85"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 37: Vigoss three-quarter length denims
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$86</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I85"/>
+  <dimension ref="A1:I86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3920,8 +3920,43 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>Vigoss Three-Quarter Length Denims</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr"/>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>Size 8 (waist approx. 30in), 21in inseam</t>
+        </is>
+      </c>
+      <c r="F86" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G86" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H86" s="4" t="inlineStr"/>
+      <c r="I86" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I85"/>
+  <autoFilter ref="A1:I86"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 38: True Religion women's jeans
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$87</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I86"/>
+  <dimension ref="A1:I87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3955,8 +3955,45 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>True Religion Women's Jeans</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E87" s="3" t="inlineStr"/>
+      <c r="F87" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G87" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H87" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="I87" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I86"/>
+  <autoFilter ref="A1:I87"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 39: second pair of True Religion jeans
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$88</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I87"/>
+  <dimension ref="A1:I88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3992,8 +3992,43 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>True Religion Women's Jeans</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr"/>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E88" s="3" t="inlineStr">
+        <is>
+          <t>24 (waist)</t>
+        </is>
+      </c>
+      <c r="F88" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G88" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H88" s="4" t="inlineStr"/>
+      <c r="I88" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I87"/>
+  <autoFilter ref="A1:I88"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 40: pink Ralph Lauren shirt
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$88</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$89</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I88"/>
+  <dimension ref="A1:I89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4027,8 +4027,50 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>Ralph Lauren Women's Shirt</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>Pink
+Pink marks on the front (see images)</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>Pink marks on the front (see images)</t>
+        </is>
+      </c>
+      <c r="E89" s="3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F89" s="3" t="inlineStr">
+        <is>
+          <t>Good vintage condition</t>
+        </is>
+      </c>
+      <c r="G89" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H89" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="I89" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I88"/>
+  <autoFilter ref="A1:I89"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 41: women's jeans size 00
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$89</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$90</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I89"/>
+  <dimension ref="A1:I90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4069,8 +4069,45 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>Women's Jeans (brand unclear)</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr"/>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E90" s="3" t="inlineStr">
+        <is>
+          <t>00 (US double-zero = UK 4, waist approx. 23-24in)</t>
+        </is>
+      </c>
+      <c r="F90" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G90" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H90" s="4" t="n">
+        <v>12.99</v>
+      </c>
+      <c r="I90" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I89"/>
+  <autoFilter ref="A1:I90"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 42: peach Juicy Couture bottoms
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$90</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$91</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I90"/>
+  <dimension ref="A1:I91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4106,8 +4106,47 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>Juicy Couture Bottoms</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>Peach</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="F91" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G91" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H91" s="4" t="inlineStr"/>
+      <c r="I91" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I90"/>
+  <autoFilter ref="A1:I91"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Set colour on 20 Aug item 7, revise price up to £34.99
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -2750,7 +2750,11 @@
           <t>Juicy Couture Track Jacket</t>
         </is>
       </c>
-      <c r="C56" s="3" t="inlineStr"/>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>Pink</t>
+        </is>
+      </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
           <t>None</t>
@@ -2772,7 +2776,7 @@
         </is>
       </c>
       <c r="H56" s="4" t="n">
-        <v>29.99</v>
+        <v>34.99</v>
       </c>
       <c r="I56" s="5" t="n">
         <v>46254</v>

</xml_diff>

<commit_message>
Correct 20 Aug item 7 colour to black, price back to £29.99
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -2752,7 +2752,7 @@
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Pink</t>
+          <t>Black</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
@@ -2776,7 +2776,7 @@
         </is>
       </c>
       <c r="H56" s="4" t="n">
-        <v>34.99</v>
+        <v>29.99</v>
       </c>
       <c r="I56" s="5" t="n">
         <v>46254</v>

</xml_diff>

<commit_message>
Price item 42 provisionally, add velour identification guide
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -4144,7 +4144,9 @@
           <t>VWM - Women's Y2K Mix</t>
         </is>
       </c>
-      <c r="H91" s="4" t="inlineStr"/>
+      <c r="H91" s="4" t="n">
+        <v>22.99</v>
+      </c>
       <c r="I91" s="5" t="n">
         <v>46254</v>
       </c>

</xml_diff>

<commit_message>
Add 20 Aug item 43: purple Juicy Couture track pants
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$92</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I91"/>
+  <dimension ref="A1:I92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4151,8 +4151,45 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>Juicy Couture Track Pants</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>Purple</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E92" s="3" t="inlineStr"/>
+      <c r="F92" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G92" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H92" s="4" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="I92" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I91"/>
+  <autoFilter ref="A1:I92"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 44: Silver Jeans Co. denim shorts
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$92</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$93</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I92"/>
+  <dimension ref="A1:I93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4188,8 +4188,47 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>Silver Jeans Co. Denim Shorts</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>Suki Mid Short style</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="inlineStr">
+        <is>
+          <t>Waist 31</t>
+        </is>
+      </c>
+      <c r="F93" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G93" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H93" s="4" t="inlineStr"/>
+      <c r="I93" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I92"/>
+  <autoFilter ref="A1:I93"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 20 Aug item 45: black bra 32A
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$93</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$94</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I93"/>
+  <dimension ref="A1:I94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4227,8 +4227,39 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>Women's Bra</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>32A</t>
+        </is>
+      </c>
+      <c r="F94" s="3" t="inlineStr"/>
+      <c r="G94" s="3" t="inlineStr"/>
+      <c r="H94" s="4" t="inlineStr"/>
+      <c r="I94" s="5" t="n">
+        <v>46254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I93"/>
+  <autoFilter ref="A1:I94"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Apply suggested prices to 20 Aug rows, refresh exports
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -3328,7 +3328,9 @@
           <t>VWM - Women's Y2K Mix</t>
         </is>
       </c>
-      <c r="H70" s="4" t="inlineStr"/>
+      <c r="H70" s="4" t="n">
+        <v>11.99</v>
+      </c>
       <c r="I70" s="5" t="n">
         <v>46254</v>
       </c>
@@ -3409,7 +3411,9 @@
           <t>VWM - Women's Y2K Mix</t>
         </is>
       </c>
-      <c r="H72" s="4" t="inlineStr"/>
+      <c r="H72" s="4" t="n">
+        <v>17.99</v>
+      </c>
       <c r="I72" s="5" t="n">
         <v>46254</v>
       </c>
@@ -3680,7 +3684,9 @@
           <t>VWM - Women's Y2K Mix</t>
         </is>
       </c>
-      <c r="H79" s="4" t="inlineStr"/>
+      <c r="H79" s="4" t="n">
+        <v>24.99</v>
+      </c>
       <c r="I79" s="5" t="n">
         <v>46254</v>
       </c>
@@ -3756,7 +3762,9 @@
           <t>VWM - Women's Y2K Mix</t>
         </is>
       </c>
-      <c r="H81" s="4" t="inlineStr"/>
+      <c r="H81" s="4" t="n">
+        <v>16.99</v>
+      </c>
       <c r="I81" s="5" t="n">
         <v>46254</v>
       </c>
@@ -3919,7 +3927,9 @@
           <t>VWM - Women's Y2K Mix</t>
         </is>
       </c>
-      <c r="H85" s="4" t="inlineStr"/>
+      <c r="H85" s="4" t="n">
+        <v>19.99</v>
+      </c>
       <c r="I85" s="5" t="n">
         <v>46254</v>
       </c>
@@ -3954,7 +3964,9 @@
           <t>VWM - Women's Y2K Mix</t>
         </is>
       </c>
-      <c r="H86" s="4" t="inlineStr"/>
+      <c r="H86" s="4" t="n">
+        <v>14.99</v>
+      </c>
       <c r="I86" s="5" t="n">
         <v>46254</v>
       </c>
@@ -4026,7 +4038,9 @@
           <t>VWM - Women's Y2K Mix</t>
         </is>
       </c>
-      <c r="H88" s="4" t="inlineStr"/>
+      <c r="H88" s="4" t="n">
+        <v>29.99</v>
+      </c>
       <c r="I88" s="5" t="n">
         <v>46254</v>
       </c>
@@ -4222,7 +4236,9 @@
           <t>VWM - Women's Y2K Mix</t>
         </is>
       </c>
-      <c r="H93" s="4" t="inlineStr"/>
+      <c r="H93" s="4" t="n">
+        <v>16.99</v>
+      </c>
       <c r="I93" s="5" t="n">
         <v>46254</v>
       </c>
@@ -4253,7 +4269,9 @@
       </c>
       <c r="F94" s="3" t="inlineStr"/>
       <c r="G94" s="3" t="inlineStr"/>
-      <c r="H94" s="4" t="inlineStr"/>
+      <c r="H94" s="4" t="n">
+        <v>8.99</v>
+      </c>
       <c r="I94" s="5" t="n">
         <v>46254</v>
       </c>

</xml_diff>

<commit_message>
Price final four 20 Aug rows
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -2612,7 +2612,9 @@
           <t>VWM - Women's Y2K Mix</t>
         </is>
       </c>
-      <c r="H52" s="4" t="inlineStr"/>
+      <c r="H52" s="4" t="n">
+        <v>12.99</v>
+      </c>
       <c r="I52" s="5" t="n">
         <v>46254</v>
       </c>
@@ -3068,7 +3070,7 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>Carhartt Women's Top (garment type unconfirmed)</t>
+          <t>Carhartt Women's Top</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
@@ -3097,7 +3099,9 @@
           <t>VWM - Women's Y2K Mix</t>
         </is>
       </c>
-      <c r="H64" s="4" t="inlineStr"/>
+      <c r="H64" s="4" t="n">
+        <v>16.99</v>
+      </c>
       <c r="I64" s="5" t="n">
         <v>46254</v>
       </c>
@@ -3264,7 +3268,7 @@
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>Val Mode Nightgown (exact type to confirm)</t>
+          <t>Val Mode Vintage Nightgown</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
@@ -3288,7 +3292,9 @@
           <t>VWM - Women's Y2K Mix</t>
         </is>
       </c>
-      <c r="H69" s="4" t="inlineStr"/>
+      <c r="H69" s="4" t="n">
+        <v>16.99</v>
+      </c>
       <c r="I69" s="5" t="n">
         <v>46254</v>
       </c>
@@ -3465,7 +3471,7 @@
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>Corset (item type and size to confirm)</t>
+          <t>Corset Top</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr"/>
@@ -3485,7 +3491,9 @@
           <t>VWM - Women's Y2K Mix</t>
         </is>
       </c>
-      <c r="H74" s="4" t="inlineStr"/>
+      <c r="H74" s="4" t="n">
+        <v>14.99</v>
+      </c>
       <c r="I74" s="5" t="n">
         <v>46254</v>
       </c>

</xml_diff>

<commit_message>
Start 21 Aug: add item 1, Tommy Hilfiger polo
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$94</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$95</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I94"/>
+  <dimension ref="A1:I95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4284,8 +4284,45 @@
         <v>46254</v>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B95" s="7" t="inlineStr">
+        <is>
+          <t>Tommy Hilfiger Polo</t>
+        </is>
+      </c>
+      <c r="C95" s="7" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="D95" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E95" s="7" t="inlineStr">
+        <is>
+          <t>Large Men's</t>
+        </is>
+      </c>
+      <c r="F95" s="7" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G95" s="7" t="inlineStr"/>
+      <c r="H95" s="8" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="I95" s="9" t="n">
+        <v>46255</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I94"/>
+  <autoFilter ref="A1:I95"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 21 Aug item 2: Fay men's top
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$96</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I95"/>
+  <dimension ref="A1:I96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4321,8 +4321,45 @@
         <v>46255</v>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>Fay Men's Top (garment type not stated)</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>Coral</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>Medium Men's</t>
+        </is>
+      </c>
+      <c r="F96" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G96" s="3" t="inlineStr"/>
+      <c r="H96" s="4" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="I96" s="5" t="n">
+        <v>46255</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I95"/>
+  <autoFilter ref="A1:I96"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Start 2 Sep: add item 1, Daisy Fuentes nightdress
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$96</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$97</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I96"/>
+  <dimension ref="A1:I97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4358,8 +4358,49 @@
         <v>46255</v>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B97" s="7" t="inlineStr">
+        <is>
+          <t>Daisy Fuentes Nightdress</t>
+        </is>
+      </c>
+      <c r="C97" s="7" t="inlineStr">
+        <is>
+          <t>Pink, 90% polyester / 10% elastane</t>
+        </is>
+      </c>
+      <c r="D97" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E97" s="7" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="F97" s="7" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G97" s="7" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="H97" s="8" t="n">
+        <v>12.99</v>
+      </c>
+      <c r="I97" s="9" t="n">
+        <v>46267</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I96"/>
+  <autoFilter ref="A1:I97"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 2 Sep item 2: Versace dress shirt
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$97</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$98</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I97"/>
+  <dimension ref="A1:I98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4399,8 +4399,49 @@
         <v>46267</v>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>Versace Business Fit Dress Shirt</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="inlineStr">
+        <is>
+          <t>Collar 16in / 41cm (approx. Large)</t>
+        </is>
+      </c>
+      <c r="F98" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G98" s="3" t="inlineStr">
+        <is>
+          <t>SF - Men's Summer Designer Mix</t>
+        </is>
+      </c>
+      <c r="H98" s="4" t="n">
+        <v>39.99</v>
+      </c>
+      <c r="I98" s="5" t="n">
+        <v>46267</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I97"/>
+  <autoFilter ref="A1:I98"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 2 Sep item 3: Nike track jacket
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$98</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$99</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I98"/>
+  <dimension ref="A1:I99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4440,8 +4440,45 @@
         <v>46267</v>
       </c>
     </row>
+    <row r="99">
+      <c r="A99" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>Nike Track Jacket</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr"/>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E99" s="3" t="inlineStr">
+        <is>
+          <t>Medium Men's</t>
+        </is>
+      </c>
+      <c r="F99" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G99" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Windbreakers</t>
+        </is>
+      </c>
+      <c r="H99" s="4" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="I99" s="5" t="n">
+        <v>46267</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I98"/>
+  <autoFilter ref="A1:I99"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 2 Sep item 4: Ralph Lauren mesh mini polo dress
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$99</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$100</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I99"/>
+  <dimension ref="A1:I100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4477,8 +4477,50 @@
         <v>46267</v>
       </c>
     </row>
+    <row r="100">
+      <c r="A100" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>Ralph Lauren Mesh Mini Polo Dress</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>Mesh mini
+Very small minor discrepancy on the front</t>
+        </is>
+      </c>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>Very small minor discrepancy on the front</t>
+        </is>
+      </c>
+      <c r="E100" s="3" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
+      <c r="F100" s="3" t="inlineStr">
+        <is>
+          <t>Very good vintage condition</t>
+        </is>
+      </c>
+      <c r="G100" s="3" t="inlineStr">
+        <is>
+          <t>VWM - RL Lacoste Polos</t>
+        </is>
+      </c>
+      <c r="H100" s="4" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="I100" s="5" t="n">
+        <v>46267</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I99"/>
+  <autoFilter ref="A1:I100"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 2 Sep item 5: Nike windbreaker
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$101</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I100"/>
+  <dimension ref="A1:I101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4519,8 +4519,46 @@
         <v>46267</v>
       </c>
     </row>
+    <row r="101">
+      <c r="A101" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B101" s="3" t="inlineStr">
+        <is>
+          <t>Nike Windbreaker</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>Black and blue, pullover style
+A couple of white marks on the front and a couple of discrepancies (see images)</t>
+        </is>
+      </c>
+      <c r="D101" s="3" t="inlineStr">
+        <is>
+          <t>A couple of white marks on the front and a couple of discrepancies (see images)</t>
+        </is>
+      </c>
+      <c r="E101" s="3" t="inlineStr"/>
+      <c r="F101" s="3" t="inlineStr">
+        <is>
+          <t>Very good vintage condition</t>
+        </is>
+      </c>
+      <c r="G101" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Windbreakers</t>
+        </is>
+      </c>
+      <c r="H101" s="4" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="I101" s="5" t="n">
+        <v>46267</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I100"/>
+  <autoFilter ref="A1:I101"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 2 Sep item 6: Lacoste women's jumper
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$102</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I101"/>
+  <dimension ref="A1:I102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4557,8 +4557,49 @@
         <v>46267</v>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>Lacoste Women's Jumper</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E102" s="3" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="F102" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G102" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Lacoste Jumpers/Cardigans</t>
+        </is>
+      </c>
+      <c r="H102" s="4" t="n">
+        <v>16.99</v>
+      </c>
+      <c r="I102" s="5" t="n">
+        <v>46267</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I101"/>
+  <autoFilter ref="A1:I102"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 2 Sep item 7: Lacoste men's polo
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$102</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$103</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I102"/>
+  <dimension ref="A1:I103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4598,8 +4598,49 @@
         <v>46267</v>
       </c>
     </row>
+    <row r="103">
+      <c r="A103" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B103" s="3" t="inlineStr">
+        <is>
+          <t>Lacoste Polo</t>
+        </is>
+      </c>
+      <c r="C103" s="3" t="inlineStr">
+        <is>
+          <t>100% cotton</t>
+        </is>
+      </c>
+      <c r="D103" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E103" s="3" t="inlineStr">
+        <is>
+          <t>XL Men's</t>
+        </is>
+      </c>
+      <c r="F103" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G103" s="3" t="inlineStr">
+        <is>
+          <t>VWM - RL Lacoste Polos</t>
+        </is>
+      </c>
+      <c r="H103" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="I103" s="5" t="n">
+        <v>46267</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I102"/>
+  <autoFilter ref="A1:I103"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Accept Offers column, set from price threshold at £20
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$J$103</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$103</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J103"/>
+  <dimension ref="A1:K103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -501,7 +501,8 @@
     <col width="26" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -552,6 +553,11 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>Accept Offers</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Date Added</t>
         </is>
       </c>
@@ -594,7 +600,12 @@
       <c r="I2" s="4" t="n">
         <v>9.99</v>
       </c>
-      <c r="J2" s="5" t="n">
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="n">
         <v>46248</v>
       </c>
     </row>
@@ -636,7 +647,12 @@
       <c r="I3" s="4" t="n">
         <v>14.99</v>
       </c>
-      <c r="J3" s="5" t="n">
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="n">
         <v>46248</v>
       </c>
     </row>
@@ -682,7 +698,12 @@
       <c r="I4" s="4" t="n">
         <v>14.99</v>
       </c>
-      <c r="J4" s="5" t="n">
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="n">
         <v>46248</v>
       </c>
     </row>
@@ -728,7 +749,12 @@
       <c r="I5" s="4" t="n">
         <v>12.99</v>
       </c>
-      <c r="J5" s="5" t="n">
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="n">
         <v>46248</v>
       </c>
     </row>
@@ -774,7 +800,12 @@
       <c r="I6" s="4" t="n">
         <v>12.99</v>
       </c>
-      <c r="J6" s="5" t="n">
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="n">
         <v>46248</v>
       </c>
     </row>
@@ -820,7 +851,12 @@
       <c r="I7" s="4" t="n">
         <v>8.99</v>
       </c>
-      <c r="J7" s="5" t="n">
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="n">
         <v>46248</v>
       </c>
     </row>
@@ -866,7 +902,12 @@
       <c r="I8" s="4" t="n">
         <v>12.99</v>
       </c>
-      <c r="J8" s="5" t="n">
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="n">
         <v>46248</v>
       </c>
     </row>
@@ -912,7 +953,12 @@
       <c r="I9" s="4" t="n">
         <v>24.99</v>
       </c>
-      <c r="J9" s="5" t="n">
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="n">
         <v>46248</v>
       </c>
     </row>
@@ -958,7 +1004,12 @@
       <c r="I10" s="4" t="n">
         <v>14.99</v>
       </c>
-      <c r="J10" s="5" t="n">
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="n">
         <v>46248</v>
       </c>
     </row>
@@ -1005,7 +1056,12 @@
       <c r="I11" s="4" t="n">
         <v>9.99</v>
       </c>
-      <c r="J11" s="5" t="n">
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="n">
         <v>46248</v>
       </c>
     </row>
@@ -1052,7 +1108,12 @@
       <c r="I12" s="4" t="n">
         <v>14.99</v>
       </c>
-      <c r="J12" s="5" t="n">
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="n">
         <v>46248</v>
       </c>
     </row>
@@ -1099,7 +1160,12 @@
       <c r="I13" s="4" t="n">
         <v>9.99</v>
       </c>
-      <c r="J13" s="5" t="n">
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="n">
         <v>46248</v>
       </c>
     </row>
@@ -1146,7 +1212,12 @@
       <c r="I14" s="4" t="n">
         <v>9.99</v>
       </c>
-      <c r="J14" s="5" t="n">
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="n">
         <v>46248</v>
       </c>
     </row>
@@ -1192,7 +1263,12 @@
       <c r="I15" s="4" t="n">
         <v>12.99</v>
       </c>
-      <c r="J15" s="5" t="n">
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="n">
         <v>46248</v>
       </c>
     </row>
@@ -1238,7 +1314,12 @@
       <c r="I16" s="4" t="n">
         <v>14.99</v>
       </c>
-      <c r="J16" s="5" t="n">
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="n">
         <v>46248</v>
       </c>
     </row>
@@ -1284,7 +1365,12 @@
       <c r="I17" s="8" t="n">
         <v>17.99</v>
       </c>
-      <c r="J17" s="9" t="n">
+      <c r="J17" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K17" s="9" t="n">
         <v>46252</v>
       </c>
     </row>
@@ -1331,7 +1417,12 @@
       <c r="I18" s="4" t="n">
         <v>17.99</v>
       </c>
-      <c r="J18" s="5" t="n">
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="n">
         <v>46252</v>
       </c>
     </row>
@@ -1373,7 +1464,12 @@
       <c r="I19" s="4" t="n">
         <v>18.99</v>
       </c>
-      <c r="J19" s="5" t="n">
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="n">
         <v>46252</v>
       </c>
     </row>
@@ -1419,7 +1515,12 @@
       <c r="I20" s="4" t="n">
         <v>18.99</v>
       </c>
-      <c r="J20" s="5" t="n">
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="n">
         <v>46252</v>
       </c>
     </row>
@@ -1465,7 +1566,12 @@
       <c r="I21" s="4" t="n">
         <v>19.99</v>
       </c>
-      <c r="J21" s="5" t="n">
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="n">
         <v>46252</v>
       </c>
     </row>
@@ -1511,7 +1617,12 @@
       <c r="I22" s="4" t="n">
         <v>14.99</v>
       </c>
-      <c r="J22" s="5" t="n">
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K22" s="5" t="n">
         <v>46252</v>
       </c>
     </row>
@@ -1553,7 +1664,12 @@
       <c r="I23" s="4" t="n">
         <v>14.99</v>
       </c>
-      <c r="J23" s="5" t="n">
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="n">
         <v>46252</v>
       </c>
     </row>
@@ -1599,7 +1715,12 @@
       <c r="I24" s="4" t="n">
         <v>27.99</v>
       </c>
-      <c r="J24" s="5" t="n">
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K24" s="5" t="n">
         <v>46252</v>
       </c>
     </row>
@@ -1646,7 +1767,12 @@
       <c r="I25" s="8" t="n">
         <v>12.99</v>
       </c>
-      <c r="J25" s="9" t="n">
+      <c r="J25" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K25" s="9" t="n">
         <v>46253</v>
       </c>
     </row>
@@ -1692,7 +1818,12 @@
       <c r="I26" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="J26" s="5" t="n">
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K26" s="5" t="n">
         <v>46253</v>
       </c>
     </row>
@@ -1738,7 +1869,12 @@
       <c r="I27" s="4" t="n">
         <v>17.99</v>
       </c>
-      <c r="J27" s="5" t="n">
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K27" s="5" t="n">
         <v>46253</v>
       </c>
     </row>
@@ -1784,7 +1920,12 @@
       <c r="I28" s="4" t="n">
         <v>14.99</v>
       </c>
-      <c r="J28" s="5" t="n">
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K28" s="5" t="n">
         <v>46253</v>
       </c>
     </row>
@@ -1826,7 +1967,12 @@
       <c r="I29" s="4" t="n">
         <v>14.99</v>
       </c>
-      <c r="J29" s="5" t="n">
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K29" s="5" t="n">
         <v>46253</v>
       </c>
     </row>
@@ -1872,7 +2018,12 @@
       <c r="I30" s="4" t="n">
         <v>13.99</v>
       </c>
-      <c r="J30" s="5" t="n">
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K30" s="5" t="n">
         <v>46253</v>
       </c>
     </row>
@@ -1918,7 +2069,12 @@
       <c r="I31" s="4" t="n">
         <v>14.99</v>
       </c>
-      <c r="J31" s="5" t="n">
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K31" s="5" t="n">
         <v>46253</v>
       </c>
     </row>
@@ -1965,7 +2121,12 @@
       <c r="I32" s="4" t="n">
         <v>13.99</v>
       </c>
-      <c r="J32" s="5" t="n">
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K32" s="5" t="n">
         <v>46253</v>
       </c>
     </row>
@@ -2012,7 +2173,12 @@
       <c r="I33" s="4" t="n">
         <v>12.99</v>
       </c>
-      <c r="J33" s="5" t="n">
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K33" s="5" t="n">
         <v>46253</v>
       </c>
     </row>
@@ -2058,7 +2224,12 @@
       <c r="I34" s="4" t="n">
         <v>14.99</v>
       </c>
-      <c r="J34" s="5" t="n">
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K34" s="5" t="n">
         <v>46253</v>
       </c>
     </row>
@@ -2104,7 +2275,12 @@
       <c r="I35" s="4" t="n">
         <v>19.99</v>
       </c>
-      <c r="J35" s="5" t="n">
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K35" s="5" t="n">
         <v>46253</v>
       </c>
     </row>
@@ -2146,7 +2322,12 @@
       <c r="I36" s="4" t="n">
         <v>14.99</v>
       </c>
-      <c r="J36" s="5" t="n">
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K36" s="5" t="n">
         <v>46253</v>
       </c>
     </row>
@@ -2192,7 +2373,12 @@
       <c r="I37" s="4" t="n">
         <v>22.99</v>
       </c>
-      <c r="J37" s="5" t="n">
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K37" s="5" t="n">
         <v>46253</v>
       </c>
     </row>
@@ -2238,7 +2424,12 @@
       <c r="I38" s="4" t="n">
         <v>12.99</v>
       </c>
-      <c r="J38" s="5" t="n">
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K38" s="5" t="n">
         <v>46253</v>
       </c>
     </row>
@@ -2280,7 +2471,12 @@
       <c r="I39" s="4" t="n">
         <v>18.99</v>
       </c>
-      <c r="J39" s="5" t="n">
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K39" s="5" t="n">
         <v>46253</v>
       </c>
     </row>
@@ -2326,7 +2522,12 @@
       <c r="I40" s="4" t="n">
         <v>19.99</v>
       </c>
-      <c r="J40" s="5" t="n">
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K40" s="5" t="n">
         <v>46253</v>
       </c>
     </row>
@@ -2372,7 +2573,12 @@
       <c r="I41" s="4" t="n">
         <v>16.99</v>
       </c>
-      <c r="J41" s="5" t="n">
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K41" s="5" t="n">
         <v>46253</v>
       </c>
     </row>
@@ -2418,7 +2624,12 @@
       <c r="I42" s="4" t="n">
         <v>34.99</v>
       </c>
-      <c r="J42" s="5" t="n">
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K42" s="5" t="n">
         <v>46253</v>
       </c>
     </row>
@@ -2465,7 +2676,12 @@
       <c r="I43" s="4" t="n">
         <v>9.99</v>
       </c>
-      <c r="J43" s="5" t="n">
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K43" s="5" t="n">
         <v>46253</v>
       </c>
     </row>
@@ -2511,7 +2727,12 @@
       <c r="I44" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="J44" s="5" t="n">
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K44" s="5" t="n">
         <v>46253</v>
       </c>
     </row>
@@ -2557,7 +2778,12 @@
       <c r="I45" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="J45" s="5" t="n">
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K45" s="5" t="n">
         <v>46253</v>
       </c>
     </row>
@@ -2603,7 +2829,12 @@
       <c r="I46" s="4" t="n">
         <v>27.99</v>
       </c>
-      <c r="J46" s="5" t="n">
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K46" s="5" t="n">
         <v>46253</v>
       </c>
     </row>
@@ -2649,7 +2880,12 @@
       <c r="I47" s="4" t="n">
         <v>24.99</v>
       </c>
-      <c r="J47" s="5" t="n">
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K47" s="5" t="n">
         <v>46253</v>
       </c>
     </row>
@@ -2691,7 +2927,12 @@
       <c r="I48" s="4" t="n">
         <v>24.99</v>
       </c>
-      <c r="J48" s="5" t="n">
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K48" s="5" t="n">
         <v>46253</v>
       </c>
     </row>
@@ -2737,7 +2978,12 @@
       <c r="I49" s="4" t="n">
         <v>24.99</v>
       </c>
-      <c r="J49" s="5" t="n">
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K49" s="5" t="n">
         <v>46253</v>
       </c>
     </row>
@@ -2784,7 +3030,12 @@
       <c r="I50" s="8" t="n">
         <v>14.99</v>
       </c>
-      <c r="J50" s="9" t="n">
+      <c r="J50" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K50" s="9" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -2830,7 +3081,12 @@
       <c r="I51" s="4" t="n">
         <v>19.99</v>
       </c>
-      <c r="J51" s="5" t="n">
+      <c r="J51" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K51" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -2876,7 +3132,12 @@
       <c r="I52" s="4" t="n">
         <v>12.99</v>
       </c>
-      <c r="J52" s="5" t="n">
+      <c r="J52" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K52" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -2923,7 +3184,12 @@
       <c r="I53" s="4" t="n">
         <v>9.99</v>
       </c>
-      <c r="J53" s="5" t="n">
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K53" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -2969,7 +3235,12 @@
       <c r="I54" s="4" t="n">
         <v>17.99</v>
       </c>
-      <c r="J54" s="5" t="n">
+      <c r="J54" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K54" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -3015,7 +3286,12 @@
       <c r="I55" s="4" t="n">
         <v>14.99</v>
       </c>
-      <c r="J55" s="5" t="n">
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K55" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -3061,7 +3337,12 @@
       <c r="I56" s="4" t="n">
         <v>29.99</v>
       </c>
-      <c r="J56" s="5" t="n">
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K56" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -3103,7 +3384,12 @@
       <c r="I57" s="4" t="n">
         <v>22.99</v>
       </c>
-      <c r="J57" s="5" t="n">
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K57" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -3149,7 +3435,12 @@
       <c r="I58" s="4" t="n">
         <v>12.99</v>
       </c>
-      <c r="J58" s="5" t="n">
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K58" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -3195,7 +3486,12 @@
       <c r="I59" s="4" t="n">
         <v>13.99</v>
       </c>
-      <c r="J59" s="5" t="n">
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K59" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -3237,7 +3533,12 @@
       <c r="I60" s="4" t="n">
         <v>19.99</v>
       </c>
-      <c r="J60" s="5" t="n">
+      <c r="J60" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K60" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -3283,7 +3584,12 @@
       <c r="I61" s="4" t="n">
         <v>12.99</v>
       </c>
-      <c r="J61" s="5" t="n">
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K61" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -3330,7 +3636,12 @@
       <c r="I62" s="4" t="n">
         <v>9.99</v>
       </c>
-      <c r="J62" s="5" t="n">
+      <c r="J62" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K62" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -3376,7 +3687,12 @@
       <c r="I63" s="4" t="n">
         <v>17.99</v>
       </c>
-      <c r="J63" s="5" t="n">
+      <c r="J63" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K63" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -3423,7 +3739,12 @@
       <c r="I64" s="4" t="n">
         <v>16.99</v>
       </c>
-      <c r="J64" s="5" t="n">
+      <c r="J64" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K64" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -3469,7 +3790,12 @@
       <c r="I65" s="4" t="n">
         <v>19.99</v>
       </c>
-      <c r="J65" s="5" t="n">
+      <c r="J65" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K65" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -3507,7 +3833,12 @@
       <c r="I66" s="4" t="n">
         <v>27.99</v>
       </c>
-      <c r="J66" s="5" t="n">
+      <c r="J66" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K66" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -3553,7 +3884,12 @@
       <c r="I67" s="4" t="n">
         <v>19.99</v>
       </c>
-      <c r="J67" s="5" t="n">
+      <c r="J67" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K67" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -3599,7 +3935,12 @@
       <c r="I68" s="4" t="n">
         <v>44.99</v>
       </c>
-      <c r="J68" s="5" t="n">
+      <c r="J68" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K68" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -3641,7 +3982,12 @@
       <c r="I69" s="4" t="n">
         <v>16.99</v>
       </c>
-      <c r="J69" s="5" t="n">
+      <c r="J69" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K69" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -3688,7 +4034,12 @@
       <c r="I70" s="4" t="n">
         <v>11.99</v>
       </c>
-      <c r="J70" s="5" t="n">
+      <c r="J70" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K70" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -3734,7 +4085,12 @@
       <c r="I71" s="4" t="n">
         <v>19.99</v>
       </c>
-      <c r="J71" s="5" t="n">
+      <c r="J71" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K71" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -3781,7 +4137,12 @@
       <c r="I72" s="4" t="n">
         <v>17.99</v>
       </c>
-      <c r="J72" s="5" t="n">
+      <c r="J72" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K72" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -3827,7 +4188,12 @@
       <c r="I73" s="4" t="n">
         <v>17.99</v>
       </c>
-      <c r="J73" s="5" t="n">
+      <c r="J73" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K73" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -3865,7 +4231,12 @@
       <c r="I74" s="4" t="n">
         <v>14.99</v>
       </c>
-      <c r="J74" s="5" t="n">
+      <c r="J74" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K74" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -3911,7 +4282,12 @@
       <c r="I75" s="4" t="n">
         <v>16.99</v>
       </c>
-      <c r="J75" s="5" t="n">
+      <c r="J75" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K75" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -3957,7 +4333,12 @@
       <c r="I76" s="4" t="n">
         <v>13.99</v>
       </c>
-      <c r="J76" s="5" t="n">
+      <c r="J76" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K76" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -4003,7 +4384,12 @@
       <c r="I77" s="4" t="n">
         <v>17.99</v>
       </c>
-      <c r="J77" s="5" t="n">
+      <c r="J77" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K77" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -4045,7 +4431,12 @@
       <c r="I78" s="4" t="n">
         <v>12.99</v>
       </c>
-      <c r="J78" s="5" t="n">
+      <c r="J78" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K78" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -4091,7 +4482,12 @@
       <c r="I79" s="4" t="n">
         <v>24.99</v>
       </c>
-      <c r="J79" s="5" t="n">
+      <c r="J79" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K79" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -4137,7 +4533,12 @@
       <c r="I80" s="4" t="n">
         <v>12.99</v>
       </c>
-      <c r="J80" s="5" t="n">
+      <c r="J80" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K80" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -4179,7 +4580,12 @@
       <c r="I81" s="4" t="n">
         <v>16.99</v>
       </c>
-      <c r="J81" s="5" t="n">
+      <c r="J81" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K81" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -4225,7 +4631,12 @@
       <c r="I82" s="4" t="n">
         <v>9.99</v>
       </c>
-      <c r="J82" s="5" t="n">
+      <c r="J82" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K82" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -4271,7 +4682,12 @@
       <c r="I83" s="4" t="n">
         <v>29.99</v>
       </c>
-      <c r="J83" s="5" t="n">
+      <c r="J83" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K83" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -4318,7 +4734,12 @@
       <c r="I84" s="4" t="n">
         <v>9.99</v>
       </c>
-      <c r="J84" s="5" t="n">
+      <c r="J84" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K84" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -4364,7 +4785,12 @@
       <c r="I85" s="4" t="n">
         <v>19.99</v>
       </c>
-      <c r="J85" s="5" t="n">
+      <c r="J85" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K85" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -4406,7 +4832,12 @@
       <c r="I86" s="4" t="n">
         <v>14.99</v>
       </c>
-      <c r="J86" s="5" t="n">
+      <c r="J86" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K86" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -4448,7 +4879,12 @@
       <c r="I87" s="4" t="n">
         <v>29.99</v>
       </c>
-      <c r="J87" s="5" t="n">
+      <c r="J87" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K87" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -4490,7 +4926,12 @@
       <c r="I88" s="4" t="n">
         <v>29.99</v>
       </c>
-      <c r="J88" s="5" t="n">
+      <c r="J88" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K88" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -4537,7 +4978,12 @@
       <c r="I89" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="J89" s="5" t="n">
+      <c r="J89" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K89" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -4579,7 +5025,12 @@
       <c r="I90" s="4" t="n">
         <v>12.99</v>
       </c>
-      <c r="J90" s="5" t="n">
+      <c r="J90" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K90" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -4625,7 +5076,12 @@
       <c r="I91" s="4" t="n">
         <v>22.99</v>
       </c>
-      <c r="J91" s="5" t="n">
+      <c r="J91" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K91" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -4667,7 +5123,12 @@
       <c r="I92" s="4" t="n">
         <v>24.99</v>
       </c>
-      <c r="J92" s="5" t="n">
+      <c r="J92" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K92" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -4713,7 +5174,12 @@
       <c r="I93" s="4" t="n">
         <v>16.99</v>
       </c>
-      <c r="J93" s="5" t="n">
+      <c r="J93" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K93" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -4751,7 +5217,12 @@
       <c r="I94" s="4" t="n">
         <v>8.99</v>
       </c>
-      <c r="J94" s="5" t="n">
+      <c r="J94" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K94" s="5" t="n">
         <v>46254</v>
       </c>
     </row>
@@ -4793,7 +5264,12 @@
       <c r="I95" s="8" t="n">
         <v>14.99</v>
       </c>
-      <c r="J95" s="9" t="n">
+      <c r="J95" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K95" s="9" t="n">
         <v>46255</v>
       </c>
     </row>
@@ -4835,7 +5311,12 @@
       <c r="I96" s="4" t="n">
         <v>19.99</v>
       </c>
-      <c r="J96" s="5" t="n">
+      <c r="J96" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K96" s="5" t="n">
         <v>46255</v>
       </c>
     </row>
@@ -4881,7 +5362,12 @@
       <c r="I97" s="8" t="n">
         <v>12.99</v>
       </c>
-      <c r="J97" s="9" t="n">
+      <c r="J97" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K97" s="9" t="n">
         <v>46267</v>
       </c>
     </row>
@@ -4927,7 +5413,12 @@
       <c r="I98" s="4" t="n">
         <v>39.99</v>
       </c>
-      <c r="J98" s="5" t="n">
+      <c r="J98" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K98" s="5" t="n">
         <v>46267</v>
       </c>
     </row>
@@ -4969,7 +5460,12 @@
       <c r="I99" s="4" t="n">
         <v>24.99</v>
       </c>
-      <c r="J99" s="5" t="n">
+      <c r="J99" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K99" s="5" t="n">
         <v>46267</v>
       </c>
     </row>
@@ -5016,7 +5512,12 @@
       <c r="I100" s="4" t="n">
         <v>14.99</v>
       </c>
-      <c r="J100" s="5" t="n">
+      <c r="J100" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K100" s="5" t="n">
         <v>46267</v>
       </c>
     </row>
@@ -5059,7 +5560,12 @@
       <c r="I101" s="4" t="n">
         <v>24.99</v>
       </c>
-      <c r="J101" s="5" t="n">
+      <c r="J101" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K101" s="5" t="n">
         <v>46267</v>
       </c>
     </row>
@@ -5105,7 +5611,12 @@
       <c r="I102" s="4" t="n">
         <v>16.99</v>
       </c>
-      <c r="J102" s="5" t="n">
+      <c r="J102" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K102" s="5" t="n">
         <v>46267</v>
       </c>
     </row>
@@ -5151,12 +5662,17 @@
       <c r="I103" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="J103" s="5" t="n">
+      <c r="J103" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K103" s="5" t="n">
         <v>46267</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J103"/>
+  <autoFilter ref="A1:K103"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Start 4 Sep: add item 1, blue Adidas windbreaker
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$103</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$104</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K103"/>
+  <dimension ref="A1:K104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5671,8 +5671,59 @@
         <v>46267</v>
       </c>
     </row>
+    <row r="104">
+      <c r="A104" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B104" s="7" t="inlineStr">
+        <is>
+          <t>Men's</t>
+        </is>
+      </c>
+      <c r="C104" s="7" t="inlineStr">
+        <is>
+          <t>Adidas Windbreaker</t>
+        </is>
+      </c>
+      <c r="D104" s="7" t="inlineStr">
+        <is>
+          <t>Blue, pullover with half zip</t>
+        </is>
+      </c>
+      <c r="E104" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F104" s="7" t="inlineStr">
+        <is>
+          <t>Large Men's</t>
+        </is>
+      </c>
+      <c r="G104" s="7" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H104" s="7" t="inlineStr">
+        <is>
+          <t>VWM - Windbreakers</t>
+        </is>
+      </c>
+      <c r="I104" s="8" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="J104" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K104" s="9" t="n">
+        <v>46269</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K103"/>
+  <autoFilter ref="A1:K104"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 4 Sep item 2: Trussardi t-shirt
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$105</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K104"/>
+  <dimension ref="A1:K105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5722,8 +5722,59 @@
         <v>46269</v>
       </c>
     </row>
+    <row r="105">
+      <c r="A105" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B105" s="3" t="inlineStr">
+        <is>
+          <t>Men's</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>Trussardi T-Shirt</t>
+        </is>
+      </c>
+      <c r="D105" s="3" t="inlineStr">
+        <is>
+          <t>Small minor discrepancy on the front</t>
+        </is>
+      </c>
+      <c r="E105" s="3" t="inlineStr">
+        <is>
+          <t>Small minor discrepancy on the front</t>
+        </is>
+      </c>
+      <c r="F105" s="3" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="G105" s="3" t="inlineStr">
+        <is>
+          <t>Very good vintage condition</t>
+        </is>
+      </c>
+      <c r="H105" s="3" t="inlineStr">
+        <is>
+          <t>SF - Men's Summer Designer Mix</t>
+        </is>
+      </c>
+      <c r="I105" s="4" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="J105" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K105" s="5" t="n">
+        <v>46269</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K104"/>
+  <autoFilter ref="A1:K105"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 4 Sep item 3: Lululemon women's hoodie
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$105</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$106</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K105"/>
+  <dimension ref="A1:K106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5773,8 +5773,59 @@
         <v>46269</v>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>Women's</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>Lululemon Women's Hoodie</t>
+        </is>
+      </c>
+      <c r="D106" s="3" t="inlineStr">
+        <is>
+          <t>Sleeve cuff slightly worn (see images)</t>
+        </is>
+      </c>
+      <c r="E106" s="3" t="inlineStr">
+        <is>
+          <t>Sleeve cuff slightly worn (see images)</t>
+        </is>
+      </c>
+      <c r="F106" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G106" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H106" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Women's Y2K Mix</t>
+        </is>
+      </c>
+      <c r="I106" s="4" t="n">
+        <v>26.99</v>
+      </c>
+      <c r="J106" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K106" s="5" t="n">
+        <v>46269</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K105"/>
+  <autoFilter ref="A1:K106"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 4 Sep item 4: cream Lacoste jumper
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$106</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$107</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K106"/>
+  <dimension ref="A1:K107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5824,8 +5824,60 @@
         <v>46269</v>
       </c>
     </row>
+    <row r="107">
+      <c r="A107" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>Unisex</t>
+        </is>
+      </c>
+      <c r="C107" s="3" t="inlineStr">
+        <is>
+          <t>Lacoste Jumper</t>
+        </is>
+      </c>
+      <c r="D107" s="3" t="inlineStr">
+        <is>
+          <t>Cream, "Chemise Lacoste" label
+Orange mark on the right shoulder (see images)</t>
+        </is>
+      </c>
+      <c r="E107" s="3" t="inlineStr">
+        <is>
+          <t>Orange mark on the right shoulder (see images)</t>
+        </is>
+      </c>
+      <c r="F107" s="3" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
+      <c r="G107" s="3" t="inlineStr">
+        <is>
+          <t>Good vintage condition</t>
+        </is>
+      </c>
+      <c r="H107" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Lacoste Jumpers/Cardigans</t>
+        </is>
+      </c>
+      <c r="I107" s="4" t="n">
+        <v>16.99</v>
+      </c>
+      <c r="J107" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K107" s="5" t="n">
+        <v>46269</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K106"/>
+  <autoFilter ref="A1:K107"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 4 Sep item 5: Izod Lacoste jumper, correct flat-price theory
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$107</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$108</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K107"/>
+  <dimension ref="A1:K108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5876,8 +5876,59 @@
         <v>46269</v>
       </c>
     </row>
+    <row r="108">
+      <c r="A108" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B108" s="3" t="inlineStr">
+        <is>
+          <t>Unisex</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>Izod Lacoste Jumper</t>
+        </is>
+      </c>
+      <c r="D108" s="3" t="inlineStr">
+        <is>
+          <t>Green, "Izod Lacoste" label</t>
+        </is>
+      </c>
+      <c r="E108" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F108" s="3" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
+      <c r="G108" s="3" t="inlineStr">
+        <is>
+          <t>Very good vintage condition</t>
+        </is>
+      </c>
+      <c r="H108" s="3" t="inlineStr">
+        <is>
+          <t>VWM - Lacoste Jumpers/Cardigans</t>
+        </is>
+      </c>
+      <c r="I108" s="4" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="J108" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K108" s="5" t="n">
+        <v>46269</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K107"/>
+  <autoFilter ref="A1:K108"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 4 Sep item 6: brown Lacoste polo, note defect wording severity
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$109</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5927,8 +5927,60 @@
         <v>46269</v>
       </c>
     </row>
+    <row r="109">
+      <c r="A109" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B109" s="3" t="inlineStr">
+        <is>
+          <t>Unisex</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>Lacoste Polo</t>
+        </is>
+      </c>
+      <c r="D109" s="3" t="inlineStr">
+        <is>
+          <t>Brown
+Slight discrepancy on the front</t>
+        </is>
+      </c>
+      <c r="E109" s="3" t="inlineStr">
+        <is>
+          <t>Slight discrepancy on the front</t>
+        </is>
+      </c>
+      <c r="F109" s="3" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
+      <c r="G109" s="3" t="inlineStr">
+        <is>
+          <t>Good condition</t>
+        </is>
+      </c>
+      <c r="H109" s="3" t="inlineStr">
+        <is>
+          <t>VWM - RL Lacoste Polos</t>
+        </is>
+      </c>
+      <c r="I109" s="4" t="n">
+        <v>12.99</v>
+      </c>
+      <c r="J109" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K109" s="5" t="n">
+        <v>46269</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K108"/>
+  <autoFilter ref="A1:K109"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 4 Sep item 7: pink Birkenstocks, resolve size premium pattern
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$109</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$110</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K109"/>
+  <dimension ref="A1:K110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5979,8 +5979,59 @@
         <v>46269</v>
       </c>
     </row>
+    <row r="110">
+      <c r="A110" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>Women's</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>Birkenstock Sandals</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>Pink</t>
+        </is>
+      </c>
+      <c r="E110" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F110" s="3" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="G110" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H110" s="3" t="inlineStr">
+        <is>
+          <t>SF - Birkenstock</t>
+        </is>
+      </c>
+      <c r="I110" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="J110" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K110" s="5" t="n">
+        <v>46269</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K109"/>
+  <autoFilter ref="A1:K110"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 4 Sep item 8: shearling Birkenstocks, style premium noted
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$110</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$111</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K110"/>
+  <dimension ref="A1:K111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6030,8 +6030,59 @@
         <v>46269</v>
       </c>
     </row>
+    <row r="111">
+      <c r="A111" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B111" s="3" t="inlineStr">
+        <is>
+          <t>Women's</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="inlineStr">
+        <is>
+          <t>Birkenstock Shearling Sandals</t>
+        </is>
+      </c>
+      <c r="D111" s="3" t="inlineStr">
+        <is>
+          <t>Black, fluffy shearling lining</t>
+        </is>
+      </c>
+      <c r="E111" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F111" s="3" t="inlineStr">
+        <is>
+          <t>37 (240mm)</t>
+        </is>
+      </c>
+      <c r="G111" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="H111" s="3" t="inlineStr">
+        <is>
+          <t>SF - Birkenstock</t>
+        </is>
+      </c>
+      <c r="I111" s="4" t="n">
+        <v>34.99</v>
+      </c>
+      <c r="J111" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K111" s="5" t="n">
+        <v>46269</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K110"/>
+  <autoFilter ref="A1:K111"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 4 Sep item 9: size 42 Birkenstocks, first filed as Men's
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$112</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K111"/>
+  <dimension ref="A1:K112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6081,8 +6081,55 @@
         <v>46269</v>
       </c>
     </row>
+    <row r="112">
+      <c r="A112" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>Men's</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>Birkenstock Sandals</t>
+        </is>
+      </c>
+      <c r="D112" s="3" t="inlineStr"/>
+      <c r="E112" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F112" s="3" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="G112" s="3" t="inlineStr">
+        <is>
+          <t>Good condition</t>
+        </is>
+      </c>
+      <c r="H112" s="3" t="inlineStr">
+        <is>
+          <t>SF - Birkenstock</t>
+        </is>
+      </c>
+      <c r="I112" s="4" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="J112" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K112" s="5" t="n">
+        <v>46269</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K111"/>
+  <autoFilter ref="A1:K112"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 4 Sep item 10: Birkenstocks, price above good-condition point
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$113</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K112"/>
+  <dimension ref="A1:K113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6128,8 +6128,51 @@
         <v>46269</v>
       </c>
     </row>
+    <row r="113">
+      <c r="A113" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B113" s="3" t="inlineStr">
+        <is>
+          <t>Unisex</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>Birkenstock Sandals</t>
+        </is>
+      </c>
+      <c r="D113" s="3" t="inlineStr"/>
+      <c r="E113" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F113" s="3" t="inlineStr"/>
+      <c r="G113" s="3" t="inlineStr">
+        <is>
+          <t>Good condition</t>
+        </is>
+      </c>
+      <c r="H113" s="3" t="inlineStr">
+        <is>
+          <t>SF - Birkenstock</t>
+        </is>
+      </c>
+      <c r="I113" s="4" t="n">
+        <v>27.99</v>
+      </c>
+      <c r="J113" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K113" s="5" t="n">
+        <v>46269</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K112"/>
+  <autoFilter ref="A1:K113"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 4 Sep item 11: size 35 Birkenstocks, completes the pricing model
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$113</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$K$114</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K113"/>
+  <dimension ref="A1:K114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6171,8 +6171,55 @@
         <v>46269</v>
       </c>
     </row>
+    <row r="114">
+      <c r="A114" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B114" s="3" t="inlineStr">
+        <is>
+          <t>Women's</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>Birkenstock Sandals</t>
+        </is>
+      </c>
+      <c r="D114" s="3" t="inlineStr"/>
+      <c r="E114" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F114" s="3" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="G114" s="3" t="inlineStr">
+        <is>
+          <t>Good condition</t>
+        </is>
+      </c>
+      <c r="H114" s="3" t="inlineStr">
+        <is>
+          <t>SF - Birkenstock</t>
+        </is>
+      </c>
+      <c r="I114" s="4" t="n">
+        <v>27.99</v>
+      </c>
+      <c r="J114" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K114" s="5" t="n">
+        <v>46269</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K113"/>
+  <autoFilter ref="A1:K114"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>